<commit_message>
Redesign the breakout around giving PMs time back
Rooms now map where the hours go, build an agent for the biggest
repetitive chunk and prove the hours it returns. Pre-work asks
participants to time their own week and plan the hours back instead
of hunting for traps; tests become Does the job / Time test / Trust
check, with the traps kept as the trust check. Story, film, kit,
readouts, slides, Pilot Pack, facilitator guide, messages and
scorecard follow the new framing. Earlier versions stay available
under ws2/archive and are linked from the kit.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q2YJhmzjoSxdfw8ZKRnAPH
</commit_message>
<xml_diff>
--- a/ws2/files/WS2_Mock_Run_Scorecard.xlsx
+++ b/ws2/files/WS2_Mock_Run_Scorecard.xlsx
@@ -1159,7 +1159,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Trap test run and the result recorded (kit-specific)</t>
+          <t>Time test run and hours back per PM per week recorded (kit-specific)</t>
         </is>
       </c>
       <c r="C18" s="11" t="n"/>
@@ -1560,7 +1560,7 @@
       </c>
       <c r="B18" s="4" t="inlineStr">
         <is>
-          <t>Trap test run and the result recorded (kit-specific)</t>
+          <t>Time test run and hours back per PM per week recorded (kit-specific)</t>
         </is>
       </c>
       <c r="C18" s="11" t="n"/>

</xml_diff>